<commit_message>
MoodleFramework integration (needs improvements)
</commit_message>
<xml_diff>
--- a/ExtensiveHealthReworkB42/Stats.xlsx
+++ b/ExtensiveHealthReworkB42/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Downloads\Mods\PZ\Custom Mods\EHR\EHR\Extensive Health Rework B42\ExtensiveHealthReworkB42\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C247C9-9F6D-4CB0-B962-2C20C3491653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4282C768-28C4-4986-B81C-36471C6FDD30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="33525" windowHeight="14355" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-17130" yWindow="2940" windowWidth="33525" windowHeight="14355" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Food Related (I guess Done)" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,9 @@
     <sheet name="Blood" sheetId="8" r:id="rId5"/>
     <sheet name="Не забыть" sheetId="5" r:id="rId6"/>
     <sheet name="Sheet1" sheetId="10" r:id="rId7"/>
-    <sheet name="RadioDialogues" sheetId="9" r:id="rId8"/>
-    <sheet name="Mechanics" sheetId="3" r:id="rId9"/>
+    <sheet name="Bugs" sheetId="11" r:id="rId8"/>
+    <sheet name="RadioDialogues" sheetId="9" r:id="rId9"/>
+    <sheet name="Mechanics" sheetId="3" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="273">
   <si>
     <t>- Cause: Rotten food (70%), burned food (5%), stale food (10%)</t>
   </si>
@@ -1138,12 +1139,54 @@
   <si>
     <t>Spiderweb bandage=1 rag, 10 spider web</t>
   </si>
+  <si>
+    <t>Не проигрывается звук чихания при фаст форварде при простуде</t>
+  </si>
+  <si>
+    <t>Проверить температуру как работает!!!</t>
+  </si>
+  <si>
+    <t>Some medications disappear when consolidate them with this mod installed I noticed this mostly with sleeping pills</t>
+  </si>
+  <si>
+    <t>when an injury heals on your character and you remove the bandage other players on MP will still see the bandage from their side</t>
+  </si>
+  <si>
+    <t>when you take medication for one of the new illnesses after you are done with the medication you still won’t get healed</t>
+  </si>
+  <si>
+    <t>the minigames like stitching needs a scaling fix</t>
+  </si>
+  <si>
+    <t>there’s some issues with food borne illnesses from non vanilla foods like vanilla foods expanded</t>
+  </si>
+  <si>
+    <t>you should add diabetes as negative trait or maybe some other diseases that are permanent as traits</t>
+  </si>
+  <si>
+    <t>Any idea why meditating (from lifestyle) produces heat?</t>
+  </si>
+  <si>
+    <t>Infection from canned food</t>
+  </si>
+  <si>
+    <t>inspecting health for other characters shows side effects multiplied infinitely, for instance mild nausea on my GFs health tab shows maybe 200 times and it keeps refreshing.</t>
+  </si>
+  <si>
+    <t> On my server, I’m using a cold environment, so I set the ambient temperature down to -20°C. The problem is that it locks my body temperature at 35.9°C no matter what I do. Even if I run in place continuously or stand right next to a fire, I can’t fully escape the hypothermia. I tried lowering the disease stage to the lowest level (stage 1 at 31°C), but I still get stuck with hypothermia at 35°C. When I turn off body temperature entirely, everything returns to normal.</t>
+  </si>
+  <si>
+    <t>Im playing on a multiplayer server without any other medical rework mods and im playing as the EHR doctor for the journal knowladge of dieseases and it seems my doc gets amnesia cause after about 5 minutes of playing i lose knowladge about all the dieseases and theres no errors to it</t>
+  </si>
+  <si>
+    <t>изменить pneumonia chance на 35%</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1301,6 +1344,24 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF7030A0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1322,7 +1383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1391,6 +1452,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2272,6 +2338,404 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53DFFC06-8A2D-4F1B-A609-E04AC1694A75}">
+  <dimension ref="B3:Z42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="14" max="14" width="11.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="C3" s="3"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
+    </row>
+    <row r="4" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B4" s="8"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="O4" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
+    </row>
+    <row r="5" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B5" s="7"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
+    </row>
+    <row r="6" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B6" s="7"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
+    </row>
+    <row r="7" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B7" s="7"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="22"/>
+      <c r="X7" s="22"/>
+    </row>
+    <row r="8" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B8" s="7"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22"/>
+      <c r="T8" s="22"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="22"/>
+      <c r="W8" s="22"/>
+      <c r="X8" s="22"/>
+    </row>
+    <row r="9" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B9" s="8"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="O9" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22"/>
+      <c r="T9" s="22"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="22"/>
+      <c r="X9" s="22"/>
+    </row>
+    <row r="10" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B10" s="8"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22"/>
+      <c r="R10" s="22"/>
+      <c r="S10" s="22"/>
+      <c r="T10" s="22"/>
+      <c r="U10" s="22"/>
+      <c r="V10" s="22"/>
+      <c r="W10" s="22"/>
+      <c r="X10" s="22"/>
+    </row>
+    <row r="11" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B11" s="7"/>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="P11" s="22"/>
+      <c r="Q11" s="22"/>
+      <c r="R11" s="22"/>
+      <c r="S11" s="22"/>
+      <c r="T11" s="22"/>
+      <c r="U11" s="22"/>
+      <c r="V11" s="22"/>
+      <c r="W11" s="22"/>
+      <c r="X11" s="22"/>
+    </row>
+    <row r="12" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B12" s="7"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="O12" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="P12" s="22"/>
+      <c r="Q12" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="R12" s="22"/>
+      <c r="S12" s="22"/>
+      <c r="T12" s="22"/>
+      <c r="U12" s="22"/>
+      <c r="V12" s="22"/>
+      <c r="W12" s="22"/>
+      <c r="X12" s="22"/>
+    </row>
+    <row r="13" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B13" s="7"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="P13" s="22"/>
+      <c r="Q13" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="R13" s="22"/>
+      <c r="S13" s="22"/>
+      <c r="T13" s="22"/>
+      <c r="U13" s="22"/>
+      <c r="V13" s="22"/>
+      <c r="W13" s="22"/>
+      <c r="X13" s="22"/>
+    </row>
+    <row r="14" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B14" s="7"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="P14" s="22"/>
+      <c r="Q14" s="22"/>
+      <c r="R14" s="22"/>
+      <c r="S14" s="22"/>
+      <c r="T14" s="22"/>
+      <c r="U14" s="22"/>
+      <c r="V14" s="22"/>
+      <c r="W14" s="22"/>
+      <c r="X14" s="22"/>
+    </row>
+    <row r="15" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B15" s="7"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="22"/>
+      <c r="Q15" s="22"/>
+      <c r="R15" s="22"/>
+      <c r="S15" s="22"/>
+      <c r="T15" s="22"/>
+      <c r="U15" s="22"/>
+      <c r="V15" s="22"/>
+      <c r="W15" s="22"/>
+      <c r="X15" s="22"/>
+    </row>
+    <row r="16" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B16" s="8"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="22"/>
+      <c r="Q16" s="22"/>
+      <c r="R16" s="22"/>
+      <c r="S16" s="22"/>
+      <c r="T16" s="22"/>
+      <c r="U16" s="22"/>
+      <c r="V16" s="22"/>
+      <c r="W16" s="22"/>
+      <c r="X16" s="22"/>
+    </row>
+    <row r="17" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B17" s="9"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="22"/>
+      <c r="Q17" s="22"/>
+      <c r="R17" s="22"/>
+      <c r="S17" s="22"/>
+      <c r="T17" s="22"/>
+      <c r="U17" s="22"/>
+      <c r="V17" s="22"/>
+      <c r="W17" s="22"/>
+      <c r="X17" s="22"/>
+    </row>
+    <row r="18" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B18" s="9"/>
+    </row>
+    <row r="19" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B19" s="9"/>
+    </row>
+    <row r="20" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="B20" s="9"/>
+    </row>
+    <row r="21" spans="2:26" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B21" s="7"/>
+    </row>
+    <row r="22" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>167</v>
+      </c>
+      <c r="E22" t="s">
+        <v>168</v>
+      </c>
+      <c r="L22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="24" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>165</v>
+      </c>
+      <c r="F24" t="s">
+        <v>166</v>
+      </c>
+      <c r="L24" t="s">
+        <v>163</v>
+      </c>
+      <c r="N24" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="26" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="S26" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="27" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="S27" t="s">
+        <v>192</v>
+      </c>
+      <c r="X27" s="3"/>
+      <c r="Z27" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="H28" t="s">
+        <v>149</v>
+      </c>
+      <c r="S28" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="S29" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="30" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="H30" t="s">
+        <v>150</v>
+      </c>
+      <c r="J30" t="s">
+        <v>151</v>
+      </c>
+      <c r="S30" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="32" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="H32" t="s">
+        <v>152</v>
+      </c>
+      <c r="I32" t="s">
+        <v>153</v>
+      </c>
+      <c r="J32" t="s">
+        <v>154</v>
+      </c>
+      <c r="S32" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="S33" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H34" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="I34" s="21"/>
+      <c r="J34" s="21" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="36" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H36" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="I36" s="22"/>
+      <c r="J36" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="K36" s="22"/>
+    </row>
+    <row r="38" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H38" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="40" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H40" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="42" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="H42" t="s">
+        <v>161</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3715F01A-79F6-4956-8F11-0E2F67879F36}">
   <dimension ref="B3:U42"/>
@@ -3570,6 +4034,192 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6582FB11-E4E7-44CC-B6AC-D03433973810}">
+  <dimension ref="B2:V21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B3" s="30" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B5" s="27" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B6" s="30" t="s">
+        <v>264</v>
+      </c>
+      <c r="V6" s="34" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B7" s="30" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B8" s="35" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B10" s="30" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B12" s="36" t="s">
+        <v>270</v>
+      </c>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="36"/>
+      <c r="L12" s="36"/>
+      <c r="M12" s="36"/>
+      <c r="N12" s="36"/>
+      <c r="O12" s="36"/>
+    </row>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="36"/>
+      <c r="L13" s="36"/>
+      <c r="M13" s="36"/>
+      <c r="N13" s="36"/>
+      <c r="O13" s="36"/>
+    </row>
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="36"/>
+      <c r="J14" s="36"/>
+      <c r="K14" s="36"/>
+      <c r="L14" s="36"/>
+      <c r="M14" s="36"/>
+      <c r="N14" s="36"/>
+      <c r="O14" s="36"/>
+    </row>
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B16" s="33" t="s">
+        <v>271</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="33"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="33"/>
+      <c r="M17" s="33"/>
+      <c r="N17" s="33"/>
+      <c r="O17" s="33"/>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="33"/>
+      <c r="K18" s="33"/>
+      <c r="L18" s="33"/>
+      <c r="M18" s="33"/>
+      <c r="N18" s="33"/>
+      <c r="O18" s="33"/>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
+      <c r="M19" s="33"/>
+      <c r="N19" s="33"/>
+      <c r="O19" s="33"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>272</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B12:O14"/>
+    <mergeCell ref="B16:O19"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21A4C555-5941-44D5-8766-80774E93DFFB}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3579,402 +4229,4 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53DFFC06-8A2D-4F1B-A609-E04AC1694A75}">
-  <dimension ref="B3:Z42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="14" max="14" width="11.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="C3" s="3"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-    </row>
-    <row r="4" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B4" s="8"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="O4" s="22" t="s">
-        <v>170</v>
-      </c>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
-    </row>
-    <row r="5" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B5" s="7"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
-      <c r="V5" s="22"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
-    </row>
-    <row r="6" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B6" s="7"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22" t="s">
-        <v>172</v>
-      </c>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="22"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="22"/>
-      <c r="V6" s="22"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="22"/>
-    </row>
-    <row r="7" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B7" s="7"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="22"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
-    </row>
-    <row r="8" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="M8" s="22"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="22" t="s">
-        <v>174</v>
-      </c>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="22"/>
-      <c r="T8" s="22"/>
-      <c r="U8" s="22"/>
-      <c r="V8" s="22"/>
-      <c r="W8" s="22"/>
-      <c r="X8" s="22"/>
-    </row>
-    <row r="9" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B9" s="8"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22" t="s">
-        <v>175</v>
-      </c>
-      <c r="O9" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="22"/>
-      <c r="S9" s="22"/>
-      <c r="T9" s="22"/>
-      <c r="U9" s="22"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="22"/>
-      <c r="X9" s="22"/>
-    </row>
-    <row r="10" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B10" s="8"/>
-      <c r="M10" s="22"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="22" t="s">
-        <v>177</v>
-      </c>
-      <c r="P10" s="22"/>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="22"/>
-      <c r="S10" s="22"/>
-      <c r="T10" s="22"/>
-      <c r="U10" s="22"/>
-      <c r="V10" s="22"/>
-      <c r="W10" s="22"/>
-      <c r="X10" s="22"/>
-    </row>
-    <row r="11" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B11" s="7"/>
-      <c r="M11" s="22"/>
-      <c r="N11" s="22"/>
-      <c r="O11" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="P11" s="22"/>
-      <c r="Q11" s="22"/>
-      <c r="R11" s="22"/>
-      <c r="S11" s="22"/>
-      <c r="T11" s="22"/>
-      <c r="U11" s="22"/>
-      <c r="V11" s="22"/>
-      <c r="W11" s="22"/>
-      <c r="X11" s="22"/>
-    </row>
-    <row r="12" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B12" s="7"/>
-      <c r="M12" s="22"/>
-      <c r="N12" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="O12" s="22" t="s">
-        <v>178</v>
-      </c>
-      <c r="P12" s="22"/>
-      <c r="Q12" s="22" t="s">
-        <v>179</v>
-      </c>
-      <c r="R12" s="22"/>
-      <c r="S12" s="22"/>
-      <c r="T12" s="22"/>
-      <c r="U12" s="22"/>
-      <c r="V12" s="22"/>
-      <c r="W12" s="22"/>
-      <c r="X12" s="22"/>
-    </row>
-    <row r="13" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B13" s="7"/>
-      <c r="M13" s="22"/>
-      <c r="N13" s="22"/>
-      <c r="O13" s="22" t="s">
-        <v>182</v>
-      </c>
-      <c r="P13" s="22"/>
-      <c r="Q13" s="22" t="s">
-        <v>180</v>
-      </c>
-      <c r="R13" s="22"/>
-      <c r="S13" s="22"/>
-      <c r="T13" s="22"/>
-      <c r="U13" s="22"/>
-      <c r="V13" s="22"/>
-      <c r="W13" s="22"/>
-      <c r="X13" s="22"/>
-    </row>
-    <row r="14" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B14" s="7"/>
-      <c r="M14" s="22"/>
-      <c r="N14" s="22"/>
-      <c r="O14" s="22" t="s">
-        <v>183</v>
-      </c>
-      <c r="P14" s="22"/>
-      <c r="Q14" s="22"/>
-      <c r="R14" s="22"/>
-      <c r="S14" s="22"/>
-      <c r="T14" s="22"/>
-      <c r="U14" s="22"/>
-      <c r="V14" s="22"/>
-      <c r="W14" s="22"/>
-      <c r="X14" s="22"/>
-    </row>
-    <row r="15" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B15" s="7"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="22"/>
-      <c r="R15" s="22"/>
-      <c r="S15" s="22"/>
-      <c r="T15" s="22"/>
-      <c r="U15" s="22"/>
-      <c r="V15" s="22"/>
-      <c r="W15" s="22"/>
-      <c r="X15" s="22"/>
-    </row>
-    <row r="16" spans="2:24" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B16" s="8"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="22"/>
-      <c r="P16" s="22"/>
-      <c r="Q16" s="22"/>
-      <c r="R16" s="22"/>
-      <c r="S16" s="22"/>
-      <c r="T16" s="22"/>
-      <c r="U16" s="22"/>
-      <c r="V16" s="22"/>
-      <c r="W16" s="22"/>
-      <c r="X16" s="22"/>
-    </row>
-    <row r="17" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B17" s="9"/>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="22"/>
-      <c r="P17" s="22"/>
-      <c r="Q17" s="22"/>
-      <c r="R17" s="22"/>
-      <c r="S17" s="22"/>
-      <c r="T17" s="22"/>
-      <c r="U17" s="22"/>
-      <c r="V17" s="22"/>
-      <c r="W17" s="22"/>
-      <c r="X17" s="22"/>
-    </row>
-    <row r="18" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B18" s="9"/>
-    </row>
-    <row r="19" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B19" s="9"/>
-    </row>
-    <row r="20" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B20" s="9"/>
-    </row>
-    <row r="21" spans="2:26" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B21" s="7"/>
-    </row>
-    <row r="22" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="C22" t="s">
-        <v>167</v>
-      </c>
-      <c r="E22" t="s">
-        <v>168</v>
-      </c>
-      <c r="L22" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="24" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="C24" t="s">
-        <v>165</v>
-      </c>
-      <c r="F24" t="s">
-        <v>166</v>
-      </c>
-      <c r="L24" t="s">
-        <v>163</v>
-      </c>
-      <c r="N24" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="26" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="S26" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="27" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="S27" t="s">
-        <v>192</v>
-      </c>
-      <c r="X27" s="3"/>
-      <c r="Z27" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="28" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="H28" t="s">
-        <v>149</v>
-      </c>
-      <c r="S28" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="29" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="S29" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="30" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="H30" t="s">
-        <v>150</v>
-      </c>
-      <c r="J30" t="s">
-        <v>151</v>
-      </c>
-      <c r="S30" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="32" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="H32" t="s">
-        <v>152</v>
-      </c>
-      <c r="I32" t="s">
-        <v>153</v>
-      </c>
-      <c r="J32" t="s">
-        <v>154</v>
-      </c>
-      <c r="S32" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="33" spans="8:19" x14ac:dyDescent="0.25">
-      <c r="S33" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="34" spans="8:19" x14ac:dyDescent="0.25">
-      <c r="H34" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="I34" s="21"/>
-      <c r="J34" s="21" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="36" spans="8:19" x14ac:dyDescent="0.25">
-      <c r="H36" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="K36" s="22"/>
-    </row>
-    <row r="38" spans="8:19" x14ac:dyDescent="0.25">
-      <c r="H38" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="40" spans="8:19" x14ac:dyDescent="0.25">
-      <c r="H40" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="42" spans="8:19" x14ac:dyDescent="0.25">
-      <c r="H42" t="s">
-        <v>161</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Moodles and HeatExposure start/end
</commit_message>
<xml_diff>
--- a/ExtensiveHealthReworkB42/Stats.xlsx
+++ b/ExtensiveHealthReworkB42/Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Downloads\Mods\PZ\Custom Mods\EHR\EHR\Extensive Health Rework B42\ExtensiveHealthReworkB42\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4282C768-28C4-4986-B81C-36471C6FDD30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865B0CF1-497F-46B6-B652-FE2C6DC82974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-17130" yWindow="2940" windowWidth="33525" windowHeight="14355" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="274">
   <si>
     <t>- Cause: Rotten food (70%), burned food (5%), stale food (10%)</t>
   </si>
@@ -1180,6 +1180,9 @@
   </si>
   <si>
     <t>изменить pneumonia chance на 35%</t>
+  </si>
+  <si>
+    <t>?? Врод еработает</t>
   </si>
 </sst>
 </file>
@@ -4042,6 +4045,9 @@
       <c r="B2" t="s">
         <v>259</v>
       </c>
+      <c r="I2" t="s">
+        <v>273</v>
+      </c>
       <c r="Q2" t="s">
         <v>260</v>
       </c>

</xml_diff>

<commit_message>
Medication Administer Fix, Blood Transfusion Added
</commit_message>
<xml_diff>
--- a/ExtensiveHealthReworkB42/Stats.xlsx
+++ b/ExtensiveHealthReworkB42/Stats.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Downloads\Mods\PZ\Custom Mods\EHR\EHR\Extensive Health Rework B42\ExtensiveHealthReworkB42\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CACFA0-E514-47CB-8B91-8C5F95A5473B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C5B2376-A2E5-4CC8-B33F-1E6EED63E6D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="2385" windowWidth="33525" windowHeight="14355" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1110" yWindow="6525" windowWidth="33525" windowHeight="14355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Food Related (I guess Done)" sheetId="1" r:id="rId1"/>
-    <sheet name="Corpse sickness (IGDnewMechanic" sheetId="2" r:id="rId2"/>
-    <sheet name="Wound Infections" sheetId="6" r:id="rId3"/>
-    <sheet name="Environmental " sheetId="7" r:id="rId4"/>
-    <sheet name="Blood" sheetId="8" r:id="rId5"/>
-    <sheet name="Не забыть" sheetId="5" r:id="rId6"/>
-    <sheet name="Sheet1" sheetId="10" r:id="rId7"/>
-    <sheet name="Bugs" sheetId="11" r:id="rId8"/>
-    <sheet name="RadioDialogues" sheetId="9" r:id="rId9"/>
-    <sheet name="Mechanics" sheetId="3" r:id="rId10"/>
+    <sheet name="TODO" sheetId="12" r:id="rId1"/>
+    <sheet name="Food Related (I guess Done)" sheetId="1" r:id="rId2"/>
+    <sheet name="Corpse sickness (IGDnewMechanic" sheetId="2" r:id="rId3"/>
+    <sheet name="Wound Infections" sheetId="6" r:id="rId4"/>
+    <sheet name="Environmental " sheetId="7" r:id="rId5"/>
+    <sheet name="Blood" sheetId="8" r:id="rId6"/>
+    <sheet name="Не забыть" sheetId="5" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="10" r:id="rId8"/>
+    <sheet name="Bugs" sheetId="11" r:id="rId9"/>
+    <sheet name="RadioDialogues" sheetId="9" r:id="rId10"/>
+    <sheet name="Mechanics" sheetId="3" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="295">
   <si>
     <t>- Cause: Rotten food (70%), burned food (5%), stale food (10%)</t>
   </si>
@@ -1189,6 +1190,110 @@
   </si>
   <si>
     <t>debugFoodPoisoning=false</t>
+  </si>
+  <si>
+    <t>Progression of diseaseses keep progressing when offline</t>
+  </si>
+  <si>
+    <t>Consolidation all problems</t>
+  </si>
+  <si>
+    <t>Consolidating items such as the antibiotic ointment and cough syrup will bug out and remove the itme, but it will return after relogging.</t>
+  </si>
+  <si>
+    <t>Not sure if it's a bug or just desync hence why I'm putting it here but in multiplayer both me and my friend have different illness whenever checking him. He has gastrointeritus where as I see he has dystery, I see an infected hand whereas he doesn't. Hard to tell what is actually to worry about.</t>
+  </si>
+  <si>
+    <t>hi I found bug I think... I playing in MP with my friend. We have a doctor. I have insomnia and I can't sleep if I don't take a sleep pills, but I take it and nothing happens but when the doctor forces to me to take it it works and I can see "active mediaction" but when I take those pills "active medication" shows nothing...</t>
+  </si>
+  <si>
+    <t>Vanilla meds not work?</t>
+  </si>
+  <si>
+    <t>What exactly happened: I'm not sure what's going on, but the painkillers aren't working for me. I take the pill, the dose is consumed, but there's no sign of any effect—neither on the panel interface, nor on the icons on the right, nor any pain relief
+-What steps did you take: took the painkillers to relieve the pain; the pill bottle; took a pill
+-MP or single-player: SP. Вот этот коммент с подозрением надо посмотреть, скорее всего там все ок</t>
+  </si>
+  <si>
+    <t>When tryingn to stitch friend in self hosted multiplayer, the mini game window that opens immediately disappears</t>
+  </si>
+  <si>
+    <t>Тоже проверить действительно ли так или просто дистанция большая</t>
+  </si>
+  <si>
+    <t>MP,
+Washing hands
+[10-08-26 00:10:57.325] ERROR: General f:570474 st:34,309,308 at KahluaThread.flushErrorMessage &gt; dumping Lua stack trace
+-----------------------------------------
+STACK TRACE
+-----------------------------------------
+Lua((MOD:Extensive Health Rework Evolved B42)).update(EHR_WashHands.lua:184).
+[10-08-26 00:10:57.325] ERROR: General f:570474 st:34,309,308&gt; Lua((MOD:Extensive Health Rework Evolved B42)).update&gt; Exception thrown
+java.lang.IllegalStateException: Forward Direction cannot be zero length vector. at IsoGameCharacter.setForwardDirection(IsoGameCharacter.java:2827).
+Stack trace:
+zombie.characters.IsoGameCharacter.setForwardDirection(IsoGameCharacter.java:2827)
+zombie.characters.IsoGameCharacter.setForwardDirection(IsoGameCharacter.java:2808)
+zombie.characters.IsoGameCharacter.faceThisObjectAlt(IsoGameCharacter.java:10609)
+java.base/jdk.internal.reflect.DirectMethodHandleAccessor.invoke(Unknown Source)
+java.base/java.lang.reflect.Method.invoke(Unknown Source)
+se.krka.kahlua.integration.expose.caller.MethodCaller.call(MethodCaller.java:58)
+se.krka.kahlua.integration.expose.LuaJavaInvoker.call(LuaJavaInvoker.java:194)
+se.krka.kahlua.integration.expose.LuaJavaInvoker.call(LuaJavaInvoker.java:184)
+se.krka.kahlua.vm.KahluaThread.callJava(KahluaThread.java:178)
+Lua((MOD:Extensive Health Rework Evolved B42)).update(EHR_WashHands.lua:184)
+se.krka.kahlua.vm.KahluaThread.luaMainloop(KahluaThread.java:795)
+se.krka.kahlua.vm.KahluaThread.call(KahluaThread.java:162)
+se.krka.kahlua.vm.KahluaThread.pcall(KahluaThread.java:1740)
+se.krka.kahlua.vm.KahluaThread.pcallvoid(KahluaThread.java:1584)
+se.krka.kahlua.integration.LuaCaller.pcallvoid(LuaCaller.java:35)
+zombie.characters.CharacterTimedActions.LuaTimedActionNew.update(LuaTimedActionNew.java:87)
+zombie.characters.IsoGameCharacter.updateInternal(IsoGameCharacter.java:9189)
+zombie.characters.IsoGameCharacter.update(IsoGameCharacter.java:8820)
+zombie.characters.IsoPlayer.updateInternal1(IsoPlayer.java:2206)
+zombie.characters.IsoPlayer.update(IsoPlayer.java:2184)
+zombie.MovingObjectUpdateSchedulerUpdateBucket.update(MovingObjectUpdateSchedulerUpdateBucket.java:58)
+zombie.MovingObjectUpdateScheduler.update(MovingObjectUpdateScheduler.java:150)
+zombie.iso.IsoCell.ProcessObjects(IsoCell.java:2662)
+zombie.iso.IsoCell.updateInternal(IsoCell.java:4905)
+zombie.iso.IsoCell.update(IsoCell.java:4862)
+zombie.iso.IsoWorld.updateWorld(IsoWorld.java:3336)
+zombie.iso.IsoWorld.updateInternal(IsoWorld.java:3428)
+zombie.iso.IsoWorld.update(IsoWorld.java:3361)
+zombie.gameStates.IngameState.updateInternal(IngameState.java:1505)
+zombie.gameStates.IngameState.update(IngameState.java:1325)
+zombie.gameStates.GameStateMachine.update(GameStateMachine.java:65)
+zombie.GameWindow.logic(GameWindow.java:390)
+zombie.GameWindow.frameStep(GameWindow.java:790)
+zombie.GameWindow.mainThreadStep(GameWindow.java:567)
+zombie.MainThread.mainLoop(MainThread.java:69)
+java.base/java.lang.Thread.run(Unknown Source)</t>
+  </si>
+  <si>
+    <t>Antidepressants - dose already active (no dose at all)</t>
+  </si>
+  <si>
+    <t>Sleeping pills - dose still active if give antidepressant first</t>
+  </si>
+  <si>
+    <t>caffeine pills - сделать OTC</t>
+  </si>
+  <si>
+    <t>Добавить крафт пакетов с кровью</t>
+  </si>
+  <si>
+    <t>Добавить больше времени на то, чтобы кровь восстанавливалась</t>
+  </si>
+  <si>
+    <t>Добавить обильную потерю крови при ранению в шею(если выйдет, то scratch не считать)</t>
+  </si>
+  <si>
+    <t>после конца действия - stress 90%, head pain, 1</t>
+  </si>
+  <si>
+    <t>добавить Item_Epinephrine (restore health to 75%, restore stamina to 90%, 20% increased move speed, fatigue to 0, if health is above do not decrease it)</t>
+  </si>
+  <si>
+    <t>Если использовать когда у персонажа больше 20% общего здоровья, то 50% шанс инсульта и мгновенной смерти</t>
   </si>
 </sst>
 </file>
@@ -2199,162 +2304,121 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:M67"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9A5698E-D7F9-417D-926B-EC214A1B994A}">
+  <dimension ref="B3:C27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="71" customWidth="1"/>
+    <col min="2" max="2" width="105.7109375" customWidth="1"/>
+    <col min="3" max="3" width="124.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
+      <c r="B3" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>1</v>
+      <c r="B4" t="s">
+        <v>277</v>
+      </c>
+      <c r="C4" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>3</v>
+      <c r="C6" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" t="s">
-        <v>16</v>
+      <c r="B8" t="s">
+        <v>281</v>
+      </c>
+      <c r="C8" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="C10" s="15" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>283</v>
+      </c>
+      <c r="C12" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="B14" s="15" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
-        <v>6</v>
+      <c r="B17" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
-        <v>9</v>
+      <c r="B18" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D36" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C41" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B42" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B43" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B44" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B45" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B46" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B47" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="M60" s="3"/>
-    </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B62" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="63" spans="2:13" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B63" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C63" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="64" spans="2:13" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="B64" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="65" spans="2:2" ht="33" x14ac:dyDescent="0.25">
-      <c r="B65" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="66" spans="2:2" ht="33" x14ac:dyDescent="0.25">
-      <c r="B66" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="67" spans="2:2" ht="33" x14ac:dyDescent="0.25">
-      <c r="B67" s="4" t="s">
-        <v>32</v>
+      <c r="B21" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>291</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21A4C555-5941-44D5-8766-80774E93DFFB}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="89.28515625" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53DFFC06-8A2D-4F1B-A609-E04AC1694A75}">
   <dimension ref="B3:Z42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2753,6 +2817,162 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B3:M67"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="71" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D36" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B44" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B45" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B46" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B47" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="M60" s="3"/>
+    </row>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="63" spans="2:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B63" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="64" spans="2:13" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="B64" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" ht="33" x14ac:dyDescent="0.25">
+      <c r="B65" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" ht="33" x14ac:dyDescent="0.25">
+      <c r="B66" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" ht="33" x14ac:dyDescent="0.25">
+      <c r="B67" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3715F01A-79F6-4956-8F11-0E2F67879F36}">
   <dimension ref="B3:U42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2932,7 +3152,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2517986B-6F4C-42D0-BD39-2D6A74ACE8BD}">
   <dimension ref="B3:R35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3231,7 +3451,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88EED2F2-04B6-485E-917E-1A8DD36BA090}">
   <dimension ref="B3:I48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3425,7 +3645,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D345CE2-5F04-48E0-AE34-8739DA490F25}">
   <dimension ref="B3:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3549,7 +3769,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCED16C1-7749-4CB3-928F-9E4FA94C1568}">
   <dimension ref="B2:AB61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3866,7 +4086,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD7944FC-5C7A-4B02-B021-398DF4A45490}">
   <dimension ref="A1:T27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4055,7 +4275,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6582FB11-E4E7-44CC-B6AC-D03433973810}">
   <dimension ref="B2:V21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4242,16 +4462,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21A4C555-5941-44D5-8766-80774E93DFFB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="89.28515625" customWidth="1"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>